<commit_message>
Update before implementing the Blackout on Macro news 15Sep2026
</commit_message>
<xml_diff>
--- a/SIM_Results/Alpaca_Live_Ledger.xlsx
+++ b/SIM_Results/Alpaca_Live_Ledger.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1226,6 +1226,466 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-09-10 15:30:04</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>2026-09-14 10:30:04</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>491</v>
+      </c>
+      <c r="E18" t="n">
+        <v>11.31</v>
+      </c>
+      <c r="F18" t="n">
+        <v>11</v>
+      </c>
+      <c r="G18" t="n">
+        <v>11.57</v>
+      </c>
+      <c r="H18" t="n">
+        <v>127.6599999999999</v>
+      </c>
+      <c r="I18" t="n">
+        <v>2.298850574712642</v>
+      </c>
+      <c r="J18" t="n">
+        <v>36.40564175548884</v>
+      </c>
+      <c r="K18" t="n">
+        <v>-0.2258711102661053</v>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>https://www.tradingview.com/chart/QxnQNEPO/?symbol=GO</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-09-09 14:30:05</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>2026-09-14 10:30:04</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>93</v>
+      </c>
+      <c r="E19" t="n">
+        <v>131.56</v>
+      </c>
+      <c r="F19" t="n">
+        <v>130</v>
+      </c>
+      <c r="G19" t="n">
+        <v>138.05</v>
+      </c>
+      <c r="H19" t="n">
+        <v>603.5700000000008</v>
+      </c>
+      <c r="I19" t="n">
+        <v>4.933110367892984</v>
+      </c>
+      <c r="J19" t="n">
+        <v>31.64410082793071</v>
+      </c>
+      <c r="K19" t="n">
+        <v>-2.534857305203644</v>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>https://www.tradingview.com/chart/QxnQNEPO/?symbol=NOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>NWSA</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-09-08 15:30:04</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>2026-09-14 10:30:04</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>687</v>
+      </c>
+      <c r="E20" t="n">
+        <v>29.88</v>
+      </c>
+      <c r="F20" t="n">
+        <v>29</v>
+      </c>
+      <c r="G20" t="n">
+        <v>30.015</v>
+      </c>
+      <c r="H20" t="n">
+        <v>92.74500000000107</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0.4518072289156679</v>
+      </c>
+      <c r="J20" t="n">
+        <v>37.20737266523901</v>
+      </c>
+      <c r="K20" t="n">
+        <v>-0.3049598320115905</v>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>https://www.tradingview.com/chart/QxnQNEPO/?symbol=NWSA</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>TEAM</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-09-11 14:30:04</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>2026-09-14 10:30:04</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>114</v>
+      </c>
+      <c r="E21" t="n">
+        <v>179.29</v>
+      </c>
+      <c r="F21" t="n">
+        <v>174</v>
+      </c>
+      <c r="G21" t="n">
+        <v>182.395</v>
+      </c>
+      <c r="H21" t="n">
+        <v>353.9700000000021</v>
+      </c>
+      <c r="I21" t="n">
+        <v>1.731831111606904</v>
+      </c>
+      <c r="J21" t="n">
+        <v>44.32023930209636</v>
+      </c>
+      <c r="K21" t="n">
+        <v>-1.360191424779259</v>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>https://www.tradingview.com/chart/QxnQNEPO/?symbol=TEAM</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>HAL</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-09-11 14:30:04</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>2026-09-14 11:06:30</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>205</v>
+      </c>
+      <c r="E22" t="n">
+        <v>35.73</v>
+      </c>
+      <c r="F22" t="n">
+        <v>35</v>
+      </c>
+      <c r="G22" t="n">
+        <v>34.980634</v>
+      </c>
+      <c r="H22" t="n">
+        <v>-153.620029999999</v>
+      </c>
+      <c r="I22" t="n">
+        <v>-2.097301987125651</v>
+      </c>
+      <c r="J22" t="n">
+        <v>37.18148211071401</v>
+      </c>
+      <c r="K22" t="n">
+        <v>-0.3486844084353251</v>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>https://www.tradingview.com/chart/QxnQNEPO/?symbol=HAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>ARKK</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-09-14 11:30:04</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>2026-09-14 12:30:04</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>89</v>
+      </c>
+      <c r="E23" t="n">
+        <v>83.87</v>
+      </c>
+      <c r="F23" t="n">
+        <v>82</v>
+      </c>
+      <c r="G23" t="n">
+        <v>84.81</v>
+      </c>
+      <c r="H23" t="n">
+        <v>83.6599999999998</v>
+      </c>
+      <c r="I23" t="n">
+        <v>1.120782162871107</v>
+      </c>
+      <c r="J23" t="n">
+        <v>43.09857372357455</v>
+      </c>
+      <c r="K23" t="n">
+        <v>-0.4213392816933634</v>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>https://www.tradingview.com/chart/QxnQNEPO/?symbol=ARKK</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>PFE</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-09-10 14:30:04</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>2026-09-14 12:30:04</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>250</v>
+      </c>
+      <c r="E24" t="n">
+        <v>27.49</v>
+      </c>
+      <c r="F24" t="n">
+        <v>27</v>
+      </c>
+      <c r="G24" t="n">
+        <v>27.825</v>
+      </c>
+      <c r="H24" t="n">
+        <v>83.75000000000021</v>
+      </c>
+      <c r="I24" t="n">
+        <v>1.218624954528923</v>
+      </c>
+      <c r="J24" t="n">
+        <v>30.8466553663467</v>
+      </c>
+      <c r="K24" t="n">
+        <v>-0.2333613615036647</v>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>https://www.tradingview.com/chart/QxnQNEPO/?symbol=PFE</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>AWK</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026-09-14 12:30:04</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>2026-09-14 15:57:59</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>125</v>
+      </c>
+      <c r="E25" t="n">
+        <v>138.28</v>
+      </c>
+      <c r="F25" t="n">
+        <v>137</v>
+      </c>
+      <c r="G25" t="n">
+        <v>139.085</v>
+      </c>
+      <c r="H25" t="n">
+        <v>100.6250000000009</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0.5821521550477341</v>
+      </c>
+      <c r="J25" t="n">
+        <v>40.39255055967946</v>
+      </c>
+      <c r="K25" t="n">
+        <v>-0.6251524487540223</v>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>https://www.tradingview.com/chart/QxnQNEPO/?symbol=AWK</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>DEC</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026-09-11 15:57:59</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>2026-09-15 10:30:05</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>185</v>
+      </c>
+      <c r="E26" t="n">
+        <v>15.122757</v>
+      </c>
+      <c r="F26" t="n">
+        <v>14</v>
+      </c>
+      <c r="G26" t="n">
+        <v>14.99</v>
+      </c>
+      <c r="H26" t="n">
+        <v>-24.56004499999996</v>
+      </c>
+      <c r="I26" t="n">
+        <v>-0.877862416224765</v>
+      </c>
+      <c r="J26" t="n">
+        <v>37.82703392937896</v>
+      </c>
+      <c r="K26" t="n">
+        <v>-0.1481773058175655</v>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>https://www.tradingview.com/chart/QxnQNEPO/?symbol=DEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>HOOD</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026-09-15 11:30:04</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>2026-09-15 14:42:46</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>36</v>
+      </c>
+      <c r="E27" t="n">
+        <v>112.06</v>
+      </c>
+      <c r="F27" t="n">
+        <v>108</v>
+      </c>
+      <c r="G27" t="n">
+        <v>107.962222</v>
+      </c>
+      <c r="H27" t="n">
+        <v>-147.5200080000002</v>
+      </c>
+      <c r="I27" t="n">
+        <v>-3.656771372479033</v>
+      </c>
+      <c r="J27" t="n">
+        <v>42.31079945427155</v>
+      </c>
+      <c r="K27" t="n">
+        <v>-1.08962938286038</v>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>https://www.tradingview.com/chart/QxnQNEPO/?symbol=HOOD</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update before implementing the Blackout on Macro news update to run each hour 17Sep2026
</commit_message>
<xml_diff>
--- a/SIM_Results/Alpaca_Live_Ledger.xlsx
+++ b/SIM_Results/Alpaca_Live_Ledger.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L27"/>
+  <dimension ref="A1:L35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1686,6 +1686,374 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>INTC</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026-09-15 12:30:04</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>2026-09-16 10:30:04</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>36</v>
+      </c>
+      <c r="E28" t="n">
+        <v>98.12</v>
+      </c>
+      <c r="F28" t="n">
+        <v>94</v>
+      </c>
+      <c r="G28" t="n">
+        <v>101.63</v>
+      </c>
+      <c r="H28" t="n">
+        <v>126.3599999999997</v>
+      </c>
+      <c r="I28" t="n">
+        <v>3.577252344068478</v>
+      </c>
+      <c r="J28" t="n">
+        <v>44.18665097873008</v>
+      </c>
+      <c r="K28" t="n">
+        <v>-0.8496808708035388</v>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>https://www.tradingview.com/chart/QxnQNEPO/?symbol=INTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026-09-14 15:57:59</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>2026-09-16 15:05:27</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>34</v>
+      </c>
+      <c r="E29" t="n">
+        <v>136.29</v>
+      </c>
+      <c r="F29" t="n">
+        <v>132</v>
+      </c>
+      <c r="G29" t="n">
+        <v>131.956471</v>
+      </c>
+      <c r="H29" t="n">
+        <v>-147.339986</v>
+      </c>
+      <c r="I29" t="n">
+        <v>-3.179638271333186</v>
+      </c>
+      <c r="J29" t="n">
+        <v>47.86802238220059</v>
+      </c>
+      <c r="K29" t="n">
+        <v>-0.6910912131309601</v>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>https://www.tradingview.com/chart/QxnQNEPO/?symbol=C</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>NEM</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-09-15 12:30:04</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>2026-09-16 14:37:10</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>93</v>
+      </c>
+      <c r="E30" t="n">
+        <v>122.6</v>
+      </c>
+      <c r="F30" t="n">
+        <v>121</v>
+      </c>
+      <c r="G30" t="n">
+        <v>120.96</v>
+      </c>
+      <c r="H30" t="n">
+        <v>-152.52</v>
+      </c>
+      <c r="I30" t="n">
+        <v>-1.33768352365416</v>
+      </c>
+      <c r="J30" t="n">
+        <v>38.70994895200425</v>
+      </c>
+      <c r="K30" t="n">
+        <v>-1.368789666804034</v>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>https://www.tradingview.com/chart/QxnQNEPO/?symbol=NEM</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>MRK</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2026-09-15 11:30:04</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>2026-09-16 15:58:00</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>144</v>
+      </c>
+      <c r="E31" t="n">
+        <v>143.58</v>
+      </c>
+      <c r="F31" t="n">
+        <v>142</v>
+      </c>
+      <c r="G31" t="n">
+        <v>144.86</v>
+      </c>
+      <c r="H31" t="n">
+        <v>184.3200000000002</v>
+      </c>
+      <c r="I31" t="n">
+        <v>0.8914890653294337</v>
+      </c>
+      <c r="J31" t="n">
+        <v>39.01479083676741</v>
+      </c>
+      <c r="K31" t="n">
+        <v>-0.8492298467588171</v>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>https://www.tradingview.com/chart/QxnQNEPO/?symbol=MRK</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>IBIT</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2026-09-16 12:30:04</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>2026-09-17 10:30:04</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>176</v>
+      </c>
+      <c r="E32" t="n">
+        <v>42.84</v>
+      </c>
+      <c r="F32" t="n">
+        <v>42</v>
+      </c>
+      <c r="G32" t="n">
+        <v>43.525</v>
+      </c>
+      <c r="H32" t="n">
+        <v>120.5599999999991</v>
+      </c>
+      <c r="I32" t="n">
+        <v>1.598972922502323</v>
+      </c>
+      <c r="J32" t="n">
+        <v>38.8572968593399</v>
+      </c>
+      <c r="K32" t="n">
+        <v>-0.3648496883542904</v>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>https://www.tradingview.com/chart/QxnQNEPO/?symbol=IBIT</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>PFE</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2026-09-15 11:30:04</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>2026-09-17 10:30:04</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>249</v>
+      </c>
+      <c r="E33" t="n">
+        <v>27.56</v>
+      </c>
+      <c r="F33" t="n">
+        <v>27</v>
+      </c>
+      <c r="G33" t="n">
+        <v>27.67</v>
+      </c>
+      <c r="H33" t="n">
+        <v>27.39000000000074</v>
+      </c>
+      <c r="I33" t="n">
+        <v>0.3991291727140892</v>
+      </c>
+      <c r="J33" t="n">
+        <v>45.8182082683434</v>
+      </c>
+      <c r="K33" t="n">
+        <v>-0.0736580033145664</v>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>https://www.tradingview.com/chart/QxnQNEPO/?symbol=PFE</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>WBD</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2026-09-09 14:30:05</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>2026-09-17 13:30:04</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>579</v>
+      </c>
+      <c r="E34" t="n">
+        <v>28.03</v>
+      </c>
+      <c r="F34" t="n">
+        <v>27</v>
+      </c>
+      <c r="G34" t="n">
+        <v>28.235</v>
+      </c>
+      <c r="H34" t="n">
+        <v>118.694999999999</v>
+      </c>
+      <c r="I34" t="n">
+        <v>0.7313592579379176</v>
+      </c>
+      <c r="J34" t="n">
+        <v>35.54795618169234</v>
+      </c>
+      <c r="K34" t="n">
+        <v>-0.10578053614487</v>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>https://www.tradingview.com/chart/QxnQNEPO/?symbol=WBD</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>AGCO</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2026-09-17 10:30:04</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>2026-09-17 14:30:04</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>60</v>
+      </c>
+      <c r="E35" t="n">
+        <v>120.33</v>
+      </c>
+      <c r="F35" t="n">
+        <v>118</v>
+      </c>
+      <c r="G35" t="n">
+        <v>122.16</v>
+      </c>
+      <c r="H35" t="n">
+        <v>109.7999999999999</v>
+      </c>
+      <c r="I35" t="n">
+        <v>1.520817751184242</v>
+      </c>
+      <c r="J35" t="n">
+        <v>40.70261443721822</v>
+      </c>
+      <c r="K35" t="n">
+        <v>-1.112748528912988</v>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>https://www.tradingview.com/chart/QxnQNEPO/?symbol=AGCO</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>